<commit_message>
floored to 0 the ups inventory
</commit_message>
<xml_diff>
--- a/OrderbookAutomation/output/Derived_Data.xlsx
+++ b/OrderbookAutomation/output/Derived_Data.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Statistics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UPS_Inventory'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UPS_Inventory'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lookup_Keys'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MOQ_Validation'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Statistics'!$A$1:$G$2</definedName>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -447,7 +447,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Allocated</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -466,10 +466,10 @@
         <v>12384</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="D2" t="n">
-        <v>12384</v>
+        <v>12072</v>
       </c>
     </row>
     <row r="3">
@@ -491,69 +491,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>64380020101</t>
+          <t>64380018701</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21624</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
-        <v>21624</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6438016101</t>
+          <t>64380020101</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>21624</v>
       </c>
       <c r="C5" t="n">
-        <v>312</v>
+        <v>648</v>
       </c>
       <c r="D5" t="n">
-        <v>-312</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>6438018701</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-24</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6438020101</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>648</v>
-      </c>
-      <c r="D7" t="n">
-        <v>-648</v>
+        <v>20976</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -663,19 +631,19 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7</v>
+        <v>0.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>